<commit_message>
Enhance admin flow tests by updating search functionality and adding member management steps; improve placeholder text for clarity.
</commit_message>
<xml_diff>
--- a/cypress/downloads/pantilla.xlsx
+++ b/cypress/downloads/pantilla.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sophiaaristizabal/Downloads/exceles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2D0A31F-D266-054A-ADDD-50C66069981E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{799048DC-1DAC-C242-9DF2-2F112A4978AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="640" windowWidth="28480" windowHeight="16040" xr2:uid="{ABCA8981-08DB-7242-9A8A-7D1E05A903CB}"/>
+    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="15980" xr2:uid="{B9238B7E-F3B8-F340-9C37-C9073BAB0DFD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,40 +36,22 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
-    <t>asignatura</t>
+    <t>institutionalId</t>
   </si>
   <si>
-    <t>periodo</t>
+    <t>profesor</t>
   </si>
   <si>
-    <t>profesor 1</t>
-  </si>
-  <si>
-    <t>profesor 2</t>
-  </si>
-  <si>
-    <t>2025-10</t>
-  </si>
-  <si>
-    <t>claseId</t>
-  </si>
-  <si>
-    <t>participantes</t>
-  </si>
-  <si>
-    <t>2 (cantidad de estudiantes en la clase)</t>
-  </si>
-  <si>
-    <t>123456 (id de la asignatura)</t>
+    <t>estudiante</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -78,14 +60,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -110,17 +86,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -454,104 +422,23 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E827C45E-1B29-0E4A-9648-CD71D55BCC64}">
-  <dimension ref="A1:F8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EB33453-AF88-644B-826C-37DADA36F569}">
+  <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="19.1640625" customWidth="1"/>
-    <col min="3" max="3" width="22.33203125" customWidth="1"/>
-    <col min="4" max="4" width="15.1640625" customWidth="1"/>
-    <col min="5" max="5" width="14.33203125" customWidth="1"/>
-    <col min="6" max="6" width="14.5" customWidth="1"/>
+    <col min="1" max="1" width="22.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="45" x14ac:dyDescent="0.2">
-      <c r="A2" s="1">
-        <v>983738</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="1">
-        <v>111223</v>
-      </c>
-      <c r="F2" s="1">
-        <v>111225</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Implement code changes to enhance functionality and improve performance
</commit_message>
<xml_diff>
--- a/cypress/downloads/pantilla.xlsx
+++ b/cypress/downloads/pantilla.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sophiaaristizabal/Downloads/exceles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{799048DC-1DAC-C242-9DF2-2F112A4978AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DE9DE9F-D6CC-7843-96E5-D08870368341}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="15980" xr2:uid="{B9238B7E-F3B8-F340-9C37-C9073BAB0DFD}"/>
+    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="15980" xr2:uid="{48E7E6FA-2C18-D54D-8226-D7B259B3ABF2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,12 +36,51 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
-  <si>
-    <t>institutionalId</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
+  <si>
+    <t>nombre</t>
+  </si>
+  <si>
+    <t>apellido</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>idInstitucional</t>
+  </si>
+  <si>
+    <t>so.aristi@gmail.com</t>
+  </si>
+  <si>
+    <t>s1017aristizabal@gmail.com</t>
+  </si>
+  <si>
+    <t>88888888888 (son 11 digitos)</t>
+  </si>
+  <si>
+    <t>Laura</t>
+  </si>
+  <si>
+    <t>Merchan</t>
+  </si>
+  <si>
+    <t>Pedro</t>
+  </si>
+  <si>
+    <t>Puentes</t>
+  </si>
+  <si>
+    <t>administrador</t>
   </si>
   <si>
     <t>profesor</t>
+  </si>
+  <si>
+    <t>coordinador</t>
+  </si>
+  <si>
+    <t>x</t>
   </si>
   <si>
     <t>estudiante</t>
@@ -60,10 +99,12 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="Arial"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -83,14 +124,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -422,25 +465,92 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EB33453-AF88-644B-826C-37DADA36F569}">
-  <dimension ref="A1:C1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB6C3C2C-1914-2240-B0F5-6299CCD5ED75}">
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.5" customWidth="1"/>
+    <col min="1" max="1" width="29" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="19.1640625" customWidth="1"/>
+    <col min="4" max="4" width="27.5" customWidth="1"/>
+    <col min="5" max="5" width="17.33203125" customWidth="1"/>
+    <col min="6" max="6" width="12.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>1232453654</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{FE43FACB-5C4F-FE40-BD3F-57222DC08FBB}"/>
+    <hyperlink ref="D3" r:id="rId2" xr:uid="{F5E93FB0-C9DF-D541-8A14-E1CD1A8AED62}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>